<commit_message>
All assigned data insights completed
</commit_message>
<xml_diff>
--- a/dataset/analytics.xlsx
+++ b/dataset/analytics.xlsx
@@ -10,6 +10,7 @@
     <sheet name="top5customers" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="ordercountperstatus" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="revenueincategories" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="mom_revenue" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -48,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -899,4 +904,50 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>revenue_month</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>current_revenue</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>previous_revenue</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>revenue_change</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>45808.79166666666</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2242.4</v>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>